<commit_message>
Cap 4 CF - O impostor
Cap 4 CF - O impostor
</commit_message>
<xml_diff>
--- a/Claude outputs/Matriz_Carro-Forte_O_Impostor.xlsx
+++ b/Claude outputs/Matriz_Carro-Forte_O_Impostor.xlsx
@@ -1946,6 +1946,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
@@ -7850,6 +7851,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -14230,7 +14232,7 @@
       </c>
       <c r="K35" s="12" t="inlineStr">
         <is>
-          <t>G: pergunta ao Gerente (fita estreita no polegar do Gerente); V: ao Caixa Veterano (polegar do Caixa Veterano).</t>
+          <t>G: pergunta ao Gerente (fita estreita no indicador do Gerente); V: ao Caixa Veterano (indicador do Caixa Veterano).</t>
         </is>
       </c>
       <c r="L35" s="12" t="inlineStr">
@@ -19206,7 +19208,7 @@
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>Como uma gaveta pesada. Uma vez logo que o rádio chamou. Outra quase um minuto e meio depois.</t>
+          <t>Como uma gaveta pesada. Uma vez logo que o rádio chamou. Outra quase dois minutos depois, logo depois de a imagem voltar.</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
@@ -21251,7 +21253,7 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>O primeiro raspado veio logo depois da ordem. O segundo, pouco antes de a imagem voltar.</t>
+          <t>O primeiro raspado veio logo depois da ordem. O segundo, logo depois de a imagem voltar.</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
@@ -26599,7 +26601,7 @@
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>A fita vendida às seis e trinta e um tem 1,2 centímetro. A do kit de primeiros socorros da Gerência, 2,5, a mesma que o Caixa Novato usa no indicador. E há uma tira estreita no polegar do Subgerente.</t>
+          <t>A fita vendida às seis e trinta e um tem 1,2 centímetro. A do kit de primeiros socorros da Gerência, 2,5, a mesma que o Caixa Novato usa no indicador. E há uma tira estreita no indicador do Subgerente.</t>
         </is>
       </c>
       <c r="H27" s="12" t="inlineStr">
@@ -26619,7 +26621,7 @@
       </c>
       <c r="K27" s="12" t="inlineStr">
         <is>
-          <t>Variante G: ... no polegar do Gerente (tabela A3; a Variante G do Cap. 8 diz "indicador"). | Variante V: ... na base do polegar do Caixa Veterano.</t>
+          <t>Variante G: ... no indicador do Gerente (tabela A3; a Variante G do Cap. 8 diz "indicador"). | Variante V: ... no indicador do Caixa Veterano.</t>
         </is>
       </c>
       <c r="L27" s="12" t="inlineStr">
@@ -27356,7 +27358,7 @@
       <c r="S37" s="12" t="inlineStr"/>
       <c r="T37" s="12" t="inlineStr">
         <is>
-          <t>Fala do impostor (marca A9 no nome). Antes, gesto: ajeita a fita no dedo (A3; em G "indicador"/polegar, em V base do polegar).</t>
+          <t>Fala do impostor (marca A9 no nome). Antes, gesto: ajeita a fita no dedo (A3; em G "indicador"/indicador, em V base do indicador).</t>
         </is>
       </c>
     </row>
@@ -29012,7 +29014,7 @@
       </c>
       <c r="G24" s="12" t="inlineStr">
         <is>
-          <t>O que o registro desmente: o sensor da porta lateral, aberta às seis e trinta e seis, quando nenhum crachá tinha passado, e o crachá dele, às sete e dezesseis, que pretendia ser a chegada; os dígitos do cartão dele no rádio; o saque em nome dele na 0392; a fita da farmácia no polegar e a luva rasgada no cesto.</t>
+          <t>O que o registro desmente: o sensor da porta lateral, aberta às seis e trinta e seis, quando nenhum crachá tinha passado, e o crachá dele, às sete e dezesseis, que pretendia ser a chegada; os dígitos do cartão dele no rádio; o saque em nome dele na 0392; a fita da farmácia no indicador e a luva rasgada no cesto.</t>
         </is>
       </c>
       <c r="H24" s="12" t="inlineStr">
@@ -29032,7 +29034,7 @@
       </c>
       <c r="K24" s="12" t="inlineStr">
         <is>
-          <t>Variante G: "dele" = Gerente; saque do resgate da previdência; fita no indicador (Variante G) ou polegar (tabela A3); o horário do crachá não tem valor definido para a G. | Variante V: "dele" = Caixa Veterano; saque das economias da aposentadoria; fita na base do polegar; horário do crachá não definido para a V.</t>
+          <t>Variante G: "dele" = Gerente; saque do resgate da previdência; fita no indicador (Variante G) ou indicador (tabela A3); o horário do crachá não tem valor definido para a G. | Variante V: "dele" = Caixa Veterano; saque das economias da aposentadoria; fita no indicador; horário do crachá não definido para a V.</t>
         </is>
       </c>
       <c r="L24" s="12" t="inlineStr">
@@ -30385,7 +30387,7 @@
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>fita no polegar (A3), farinha na barra (A6), cartão do rádio (A7)</t>
+          <t>fita no indicador (A3), farinha na barra (A6), cartão do rádio (A7)</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
@@ -30440,7 +30442,7 @@
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>fita (A3: tabela diz polegar, Variante G diz indicador), farinha (A6), cartão (A7)</t>
+          <t>fita (A3: tabela diz indicador, Variante G diz indicador), farinha (A6), cartão (A7)</t>
         </is>
       </c>
       <c r="J3" s="9" t="inlineStr">
@@ -30495,7 +30497,7 @@
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>fita na base do polegar (A3), farinha (A6), cartão (A7)</t>
+          <t>fita no indicador (A3), farinha (A6), cartão (A7)</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
@@ -30509,6 +30511,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
@@ -30621,7 +30624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -30718,7 +30721,11 @@
           <t>Unificar: corte e fita no mesmo dedo nas três partidas (ou rasgo no polegar, ou fita no indicador). Lembrar que o Caixa Novato usa fita larga no indicador — o contraste largura 1,2 × 2,5 cm continua a pista.</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr"/>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>DECIDIDO 05/10: fita estreita no INDICADOR do impostor nas três partidas (mesmo dedo do rasgo da luva).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -30738,7 +30745,7 @@
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Pela rota, o impostor volta à Gerência às 7h59:54 (+109 s), depois de a câmera voltar (7h59:39). O Novato diz "quase um minuto e meio depois" (Cap. 4) e "pouco antes de a imagem voltar" (Cap. 5).</t>
+          <t>Pela rota, o impostor volta à Gerência às 7h59:54 (+109 s), depois de a câmera voltar (7h59:39). O Novato diz "quase dois minutos depois, logo depois de a imagem voltar" (Cap. 4) e "logo depois de a imagem voltar" (Cap. 5).</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
@@ -30746,7 +30753,11 @@
           <t>Mudar a fala para "quase dois minutos depois" / "logo depois de a imagem voltar", ou o raspado vir do fundo do Rack ao reentrar (7h59:39). A grade da janela precisa fechar antes da narração.</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr"/>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>DECIDIDO 05/10: "quase dois minutos depois, logo depois de a imagem voltar" (Caps. 4 e 5).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -30774,7 +30785,11 @@
           <t>Corrigir a tabela: "Completa" só para o Transportador; oculto e vigia "Sempre" (do sistema, nunca humanos). A matriz já segue assim.</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr"/>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>APLICADO 05/10: oculto e vigia sempre presentes, do sistema.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -30802,7 +30817,11 @@
           <t>A Operadora lê o histórico em toda casa; a Estagiária fica como reforço (ela já está na Central).</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>APLICADO 05/10 (Cap. 2): sem a Estagiária, a Operadora lê.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -30858,7 +30877,11 @@
           <t>Passar a observação à Auditora ou à Cliente do Cofre (que repara em detalhes) nas casas sem a Farmacêutica.</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>APLICADO 05/10 (Cap. 2): sem a Farmacêutica, a Auditora vê.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -30942,7 +30965,11 @@
           <t>Nas casas sem Subgerente: a sugestão do clone passa ao Caixa Veterano; a resposta dupla vira silêncio do Gerente + versão da Operadora.</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr"/>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>APLICADO 05/10 (Cap. 2): clone com o Caixa Veterano; só o Gerente responde "Manutenção".</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -30998,7 +31025,11 @@
           <t>O sensor (6h36) e a caixa de 1998 continuam fechando o ponto; a falsa pista do guarda-chuva vira exclusiva das casas de 10+.</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>APLICADO 05/10 (Cap. 4): sem o Padeiro, sai a cena do guarda-chuva.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -31167,6 +31198,70 @@
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Decisão</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Gerente humano</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Elenco; Caps. 4, 6, 7</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>O Gerente faz o encobrimento das 8h31 em toda partida.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>DECIDIDO 05/10: o Gerente é sempre do sistema (como o ajudante consciente).</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>DECIDIDO 05/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Decisão</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Pegadas sem a Limpeza</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Cap. 4</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Sem o Funcionário da Limpeza, ninguém descreve as pegadas.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>A Auditora diz a frase.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>APLICADO 05/10</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F19"/>
@@ -31272,17 +31367,17 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>No polegar do Subgerente</t>
+          <t>No indicador do Subgerente</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>No polegar do Gerente</t>
+          <t>No indicador do Gerente</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>No polegar do Caixa Veterano</t>
+          <t>No indicador do Caixa Veterano</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr"/>
@@ -36603,6 +36698,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>

</xml_diff>